<commit_message>
added backgrounds and logos
</commit_message>
<xml_diff>
--- a/ctl-site/src/assets/AEC.xlsx
+++ b/ctl-site/src/assets/AEC.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29127"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\code\ctl-angular\ctl-angular\src\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/9be54d10f24db4ff/CTL site/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{260EA5DC-4F81-4A07-BB33-3D2366529A25}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{7520A2BC-A50F-40E1-BC90-C042092A250F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1080" yWindow="1200" windowWidth="17280" windowHeight="10632" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet_1" sheetId="1" r:id="rId1"/>
@@ -24,8 +24,190 @@
 </workbook>
 </file>
 
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="17">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="1"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="2"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="3"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="4"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="5"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="6"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="7"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="8"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="9"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="10"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="11"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="12"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="13"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="14"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="15"/>
+        </ext>
+      </extLst>
+    </bk>
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="16"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="17">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+    <bk>
+      <rc t="1" v="1"/>
+    </bk>
+    <bk>
+      <rc t="1" v="2"/>
+    </bk>
+    <bk>
+      <rc t="1" v="3"/>
+    </bk>
+    <bk>
+      <rc t="1" v="4"/>
+    </bk>
+    <bk>
+      <rc t="1" v="5"/>
+    </bk>
+    <bk>
+      <rc t="1" v="6"/>
+    </bk>
+    <bk>
+      <rc t="1" v="7"/>
+    </bk>
+    <bk>
+      <rc t="1" v="8"/>
+    </bk>
+    <bk>
+      <rc t="1" v="9"/>
+    </bk>
+    <bk>
+      <rc t="1" v="10"/>
+    </bk>
+    <bk>
+      <rc t="1" v="11"/>
+    </bk>
+    <bk>
+      <rc t="1" v="12"/>
+    </bk>
+    <bk>
+      <rc t="1" v="13"/>
+    </bk>
+    <bk>
+      <rc t="1" v="14"/>
+    </bk>
+    <bk>
+      <rc t="1" v="15"/>
+    </bk>
+    <bk>
+      <rc t="1" v="16"/>
+    </bk>
+  </valueMetadata>
+</metadata>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="20">
   <si>
     <t>DESCRIÇÃO COMPLETA</t>
   </si>
@@ -49,6 +231,47 @@
   <si>
     <t>DESCRIÇÃO PEQUENA 
 (Topo da página)</t>
+  </si>
+  <si>
+    <t>Escola Básica de Almas de Freire [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Almas de Freire [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Cruz de Morouços [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Casais do Campo [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Taveiro [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Arzila [AECO]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Ameal [AECO]</t>
+  </si>
+  <si>
+    <t>O CTL desenvolve, no âmbito da sua missão educativa e social, um conjunto de Atividades de Enriquecimento Curricular (AEC) dirigidas às crianças do 1.º Ciclo do Ensino Básico. Estas atividades têm como objetivo complementar o percurso escolar, promovendo competências essenciais, o desenvolvimento integral e o bem-estar das crianças, num ambiente seguro, inclusivo e estimulante.
+As AEC do CTL são dinamizadas por profissionais qualificados e planeadas de forma a facilitar a descoberta de novas áreas de interesse, reforçar aprendizagens e proporcionar experiências diversificadas fora do contexto curricular tradicional. Através de metodologias ativas e lúdicas, incentivamos a criatividade, a autonomia, a cooperação e o respeito pelos outros.
+Entre as áreas trabalhadas encontram-se, habitualmente, a expressão artística, a atividade física e desportiva, a música, o inglês, as tecnologias, os projetos temáticos e outras iniciativas que cada ano letivo pode integrar, de acordo com as necessidades das escolas e da comunidade educativa.</t>
+  </si>
+  <si>
+    <t>Onde desenvolvemos as AEC:</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de São Bartolomeu [AECC]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica Poeta Silva Gaio [AECC]</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> - Escola Básica de Cernache [AECC]</t>
+  </si>
+  <si>
+    <t>Projeto +AEC</t>
   </si>
 </sst>
 </file>
@@ -185,6 +408,150 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="17">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>1</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>2</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>3</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>4</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>5</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>6</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>7</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>8</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>9</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>10</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>11</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>12</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>13</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>14</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>15</v>
+    <v>5</v>
+  </rv>
+  <rv s="0">
+    <v>16</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+  <rel r:id="rId2"/>
+  <rel r:id="rId3"/>
+  <rel r:id="rId4"/>
+  <rel r:id="rId5"/>
+  <rel r:id="rId6"/>
+  <rel r:id="rId7"/>
+  <rel r:id="rId8"/>
+  <rel r:id="rId9"/>
+  <rel r:id="rId10"/>
+  <rel r:id="rId11"/>
+  <rel r:id="rId12"/>
+  <rel r:id="rId13"/>
+  <rel r:id="rId14"/>
+  <rel r:id="rId15"/>
+  <rel r:id="rId16"/>
+  <rel r:id="rId17"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -451,19 +818,26 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:Z17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.88671875" style="1" customWidth="1"/>
-    <col min="2" max="2" width="52.44140625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="39.77734375" style="2" customWidth="1"/>
-    <col min="4" max="4" width="41.33203125" style="2" customWidth="1"/>
-    <col min="5" max="5" width="37.6640625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="28.21875" style="2" customWidth="1"/>
-    <col min="7" max="7" width="25.5546875" style="2" customWidth="1"/>
-    <col min="8" max="16384" width="8.88671875" style="2"/>
+    <col min="1" max="1" width="25.85546875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="62.140625" style="2" customWidth="1"/>
+    <col min="3" max="3" width="22.5703125" style="2" customWidth="1"/>
+    <col min="4" max="4" width="20.7109375" style="2" customWidth="1"/>
+    <col min="5" max="5" width="22.85546875" style="2" customWidth="1"/>
+    <col min="6" max="6" width="16.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="17" style="2" customWidth="1"/>
+    <col min="8" max="8" width="16.140625" style="2" customWidth="1"/>
+    <col min="9" max="9" width="17.7109375" style="2" customWidth="1"/>
+    <col min="10" max="10" width="17.140625" style="2" customWidth="1"/>
+    <col min="11" max="11" width="18.28515625" style="2" customWidth="1"/>
+    <col min="12" max="12" width="12.7109375" style="2" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" style="2"/>
+    <col min="14" max="14" width="10.7109375" style="2" customWidth="1"/>
+    <col min="15" max="16384" width="8.85546875" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:26" ht="33.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:26" ht="33.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>6</v>
       </c>
@@ -493,11 +867,13 @@
       <c r="Y1" s="9"/>
       <c r="Z1" s="9"/>
     </row>
-    <row r="2" spans="1:26" ht="124.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:26" ht="207.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="4"/>
+      <c r="B2" s="4" t="s">
+        <v>14</v>
+      </c>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
       <c r="E2" s="9"/>
@@ -523,11 +899,13 @@
       <c r="Y2" s="9"/>
       <c r="Z2" s="9"/>
     </row>
-    <row r="3" spans="1:26" ht="38.4" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:26" ht="38.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="5"/>
+      <c r="B3" s="5" t="s">
+        <v>15</v>
+      </c>
       <c r="C3" s="9"/>
       <c r="D3" s="9"/>
       <c r="E3" s="9"/>
@@ -553,20 +931,40 @@
       <c r="Y3" s="9"/>
       <c r="Z3" s="9"/>
     </row>
-    <row r="4" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:26" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="3"/>
-      <c r="C4" s="3"/>
-      <c r="D4" s="3"/>
-      <c r="E4" s="3"/>
-      <c r="F4" s="3"/>
-      <c r="G4" s="3"/>
-      <c r="H4" s="3"/>
-      <c r="I4" s="3"/>
-      <c r="J4" s="3"/>
-      <c r="K4" s="3"/>
+      <c r="B4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="F4" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="K4" s="3" t="s">
+        <v>18</v>
+      </c>
       <c r="L4" s="3"/>
       <c r="M4" s="3"/>
       <c r="N4" s="3"/>
@@ -583,11 +981,13 @@
       <c r="Y4" s="3"/>
       <c r="Z4" s="3"/>
     </row>
-    <row r="5" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:26" ht="27" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="8" t="s">
         <v>2</v>
       </c>
-      <c r="B5" s="5"/>
+      <c r="B5" s="5" t="s">
+        <v>19</v>
+      </c>
       <c r="C5" s="9"/>
       <c r="D5" s="9"/>
       <c r="E5" s="9"/>
@@ -613,11 +1013,13 @@
       <c r="Y5" s="9"/>
       <c r="Z5" s="9"/>
     </row>
-    <row r="6" spans="1:26" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:26" ht="42.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="3"/>
+      <c r="B6" s="3" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
       <c r="C6" s="3"/>
       <c r="D6" s="3"/>
       <c r="E6" s="3"/>
@@ -643,26 +1045,58 @@
       <c r="Y6" s="3"/>
       <c r="Z6" s="3"/>
     </row>
-    <row r="7" spans="1:26" ht="87.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:26" ht="87.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="B7" s="3"/>
-      <c r="C7" s="3"/>
-      <c r="D7" s="3"/>
-      <c r="E7" s="3"/>
-      <c r="F7" s="3"/>
-      <c r="G7" s="3"/>
-      <c r="H7" s="3"/>
-      <c r="I7" s="3"/>
-      <c r="J7" s="3"/>
-      <c r="K7" s="3"/>
-      <c r="L7" s="3"/>
-      <c r="M7" s="3"/>
-      <c r="N7" s="3"/>
-      <c r="O7" s="3"/>
-      <c r="P7" s="3"/>
-      <c r="Q7" s="3"/>
+      <c r="B7" s="3" t="e" vm="2">
+        <v>#VALUE!</v>
+      </c>
+      <c r="C7" s="3" t="e" vm="3">
+        <v>#VALUE!</v>
+      </c>
+      <c r="D7" s="3" t="e" vm="4">
+        <v>#VALUE!</v>
+      </c>
+      <c r="E7" s="3" t="e" vm="5">
+        <v>#VALUE!</v>
+      </c>
+      <c r="F7" s="3" t="e" vm="6">
+        <v>#VALUE!</v>
+      </c>
+      <c r="G7" s="3" t="e" vm="7">
+        <v>#VALUE!</v>
+      </c>
+      <c r="H7" s="3" t="e" vm="8">
+        <v>#VALUE!</v>
+      </c>
+      <c r="I7" s="3" t="e" vm="9">
+        <v>#VALUE!</v>
+      </c>
+      <c r="J7" s="3" t="e" vm="10">
+        <v>#VALUE!</v>
+      </c>
+      <c r="K7" s="3" t="e" vm="11">
+        <v>#VALUE!</v>
+      </c>
+      <c r="L7" s="3" t="e" vm="12">
+        <v>#VALUE!</v>
+      </c>
+      <c r="M7" s="3" t="e" vm="13">
+        <v>#VALUE!</v>
+      </c>
+      <c r="N7" s="3" t="e" vm="14">
+        <v>#VALUE!</v>
+      </c>
+      <c r="O7" s="3" t="e" vm="15">
+        <v>#VALUE!</v>
+      </c>
+      <c r="P7" s="3" t="e" vm="16">
+        <v>#VALUE!</v>
+      </c>
+      <c r="Q7" s="3" t="e" vm="17">
+        <v>#VALUE!</v>
+      </c>
       <c r="R7" s="3"/>
       <c r="S7" s="3"/>
       <c r="T7" s="3"/>
@@ -673,7 +1107,7 @@
       <c r="Y7" s="3"/>
       <c r="Z7" s="3"/>
     </row>
-    <row r="8" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A8" s="10"/>
       <c r="B8" s="9"/>
       <c r="C8" s="9"/>
@@ -701,7 +1135,7 @@
       <c r="Y8" s="9"/>
       <c r="Z8" s="9"/>
     </row>
-    <row r="9" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A9" s="10"/>
       <c r="B9" s="9"/>
       <c r="C9" s="9"/>
@@ -729,7 +1163,7 @@
       <c r="Y9" s="9"/>
       <c r="Z9" s="9"/>
     </row>
-    <row r="10" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A10" s="10"/>
       <c r="B10" s="9"/>
       <c r="C10" s="9"/>
@@ -757,7 +1191,7 @@
       <c r="Y10" s="9"/>
       <c r="Z10" s="9"/>
     </row>
-    <row r="11" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A11" s="10"/>
       <c r="B11" s="9"/>
       <c r="C11" s="9"/>
@@ -785,7 +1219,7 @@
       <c r="Y11" s="9"/>
       <c r="Z11" s="9"/>
     </row>
-    <row r="12" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A12" s="10"/>
       <c r="B12" s="9"/>
       <c r="C12" s="9"/>
@@ -813,7 +1247,7 @@
       <c r="Y12" s="9"/>
       <c r="Z12" s="9"/>
     </row>
-    <row r="13" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A13" s="10"/>
       <c r="B13" s="9"/>
       <c r="C13" s="9"/>
@@ -841,7 +1275,7 @@
       <c r="Y13" s="9"/>
       <c r="Z13" s="9"/>
     </row>
-    <row r="14" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A14" s="10"/>
       <c r="B14" s="9"/>
       <c r="C14" s="9"/>
@@ -869,7 +1303,7 @@
       <c r="Y14" s="9"/>
       <c r="Z14" s="9"/>
     </row>
-    <row r="15" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A15" s="10"/>
       <c r="B15" s="9"/>
       <c r="C15" s="9"/>
@@ -897,7 +1331,7 @@
       <c r="Y15" s="9"/>
       <c r="Z15" s="9"/>
     </row>
-    <row r="16" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A16" s="10"/>
       <c r="B16" s="9"/>
       <c r="C16" s="9"/>
@@ -925,7 +1359,7 @@
       <c r="Y16" s="9"/>
       <c r="Z16" s="9"/>
     </row>
-    <row r="17" spans="1:26" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:26" x14ac:dyDescent="0.25">
       <c r="A17" s="10"/>
       <c r="B17" s="9"/>
       <c r="C17" s="9"/>

</xml_diff>